<commit_message>
Coach peptides display + mobile workout detail with demo video links
- Coach Supplements tab now shows a read-only Peptides panel (peptideCycles),
  since the ProtocolEditor only reads protocolItems.
- Workouts bulk grid gains a 'Video Link' column (coach-pasted or AI-extracted),
  persisted per exercise.
- Guided/Full 'today' now lists each of today's exercises individually with
  sets x reps, rest, muscle group, and notes, plus a 'Watch demo' link when a
  video URL is set. Workout/CSV/XLSX templates updated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/workouts-template.xlsx
+++ b/public/templates/workouts-template.xlsx
@@ -397,15 +397,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:H6"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="16.83203125" customWidth="1"/>
-    <col min="5" max="5" width="16.83203125" customWidth="1"/>
-    <col min="6" max="6" width="16.83203125" customWidth="1"/>
-    <col min="7" max="7" width="42.83203125" customWidth="1"/>
+    <col min="1" max="1" width="14.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="14.83203125" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="34.83203125" customWidth="1"/>
+    <col min="8" max="8" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -430,6 +431,9 @@
       <c r="G1" t="str">
         <v>notes</v>
       </c>
+      <c r="H1" t="str">
+        <v>videoUrl</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -453,6 +457,9 @@
       <c r="G2" t="str">
         <v>Warm up thoroughly</v>
       </c>
+      <c r="H2" t="str">
+        <v>https://youtu.be/rT7DgCr-3pg</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -476,28 +483,34 @@
       <c r="G3" t="str">
         <v/>
       </c>
+      <c r="H3" t="str">
+        <v>https://youtu.be/2yjwXTZQDDI</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Day 1 - Push</v>
+        <v>Day 2 - Pull</v>
       </c>
       <c r="B4" t="str">
-        <v>Cable Fly</v>
+        <v>Deadlift</v>
       </c>
       <c r="C4" t="str">
-        <v>Chest</v>
+        <v>Back</v>
       </c>
       <c r="D4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="str">
-        <v>12-15</v>
+        <v>5</v>
       </c>
       <c r="F4">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="G4" t="str">
         <v/>
+      </c>
+      <c r="H4" t="str">
+        <v>https://youtu.be/op9kVnSso6Q</v>
       </c>
     </row>
     <row r="5">
@@ -505,73 +518,56 @@
         <v>Day 2 - Pull</v>
       </c>
       <c r="B5" t="str">
-        <v>Deadlift</v>
+        <v>Pull-Up</v>
       </c>
       <c r="C5" t="str">
         <v>Back</v>
       </c>
       <c r="D5">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E5" t="str">
-        <v>5</v>
+        <v>AMRAP</v>
       </c>
       <c r="F5">
-        <v>150</v>
+        <v>90</v>
       </c>
       <c r="G5" t="str">
-        <v/>
+        <v>Add weight if easy</v>
+      </c>
+      <c r="H5" t="str">
+        <v>https://youtu.be/eGo4IYlbE5g</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Day 2 - Pull</v>
+        <v>Day 3 - Legs</v>
       </c>
       <c r="B6" t="str">
-        <v>Pull-Up</v>
+        <v>Back Squat</v>
       </c>
       <c r="C6" t="str">
-        <v>Back</v>
+        <v>Quads</v>
       </c>
       <c r="D6">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E6" t="str">
-        <v>AMRAP</v>
+        <v>8-10</v>
       </c>
       <c r="F6">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="G6" t="str">
-        <v>Add weight if easy</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Day 3 - Legs</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Back Squat</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Quads</v>
-      </c>
-      <c r="D7">
-        <v>4</v>
-      </c>
-      <c r="E7" t="str">
-        <v>8-10</v>
-      </c>
-      <c r="F7">
-        <v>120</v>
-      </c>
-      <c r="G7" t="str">
         <v/>
+      </c>
+      <c r="H6" t="str">
+        <v>https://youtu.be/ultWZbUMPL8</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>